<commit_message>
Fill in group 6 names; extend experiment Excel with app check and iteration history
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AWLf4Vf7U3nex8wdXcBp7P
</commit_message>
<xml_diff>
--- a/ISOM5240_GroupProject/results/Experimental_results.xlsx
+++ b/ISOM5240_GroupProject/results/Experimental_results.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Confusion_segment" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_App_performance" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Error_examples" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Streamlit_Cloud_check" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Iteration_history" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,13 +35,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A5F"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -60,11 +71,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2185,4 +2197,599 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>app_model</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>where</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>test_samples</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>true_label</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>pred_1</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>pred_2</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>pred_3</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ludanzhang54/oh-review-sentiment</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Streamlit Cloud (Accuracy check tab)</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>300</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.7333</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>71</v>
+      </c>
+      <c r="H2" t="n">
+        <v>21</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>pred_1..3 = negative / neutral / positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>22</v>
+      </c>
+      <c r="H3" t="n">
+        <v>63</v>
+      </c>
+      <c r="I3" t="n">
+        <v>18</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>3</v>
+      </c>
+      <c r="H4" t="n">
+        <v>15</v>
+      </c>
+      <c r="I4" t="n">
+        <v>86</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ludanzhang54/oh-guest-segment</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Streamlit Cloud (Accuracy check tab)</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>300</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.7433</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>108</v>
+      </c>
+      <c r="H5" t="n">
+        <v>32</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>pred_1..2 = business / leisure</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>leisure</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" t="n">
+        <v>115</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Result: identical to Notebook 03, sheet 4_App_performance (same 300 reviews, seed 42): 73.33% and 74.33%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>iteration</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>task</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>labels</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>reviews_per_label</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>split</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>samples</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>macro_f1</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>negative/neutral/positive</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.7333</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.7345</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>within 0.5 pt of distilroberta -&gt; smaller model</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>negative/neutral/positive</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>distilroberta-base</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.7361</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.7377</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>negative/neutral/positive</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.7272</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.7281</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>business/couple/family</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>distilroberta-base</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1800</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.5583</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.5544</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>family recall 0.43; 202/600 family -&gt; couple</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>sentiment</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>negative/neutral/positive</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>4500</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.7496</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.7503</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>+2.2 pts vs iteration 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>business/leisure</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>distilbert-base-uncased</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.7207</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.7206</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>segments redefined; 2.5x more data</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>